<commit_message>
Fix Mythril/Echidna runners & decision_engine. Update image to mythril/myth, add VulnerableTest.sol demo contract. Docker login & pulls ready.
</commit_message>
<xml_diff>
--- a/reports/contracts_summary.xlsx
+++ b/reports/contracts_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,14 +495,586 @@
           <t>LOW</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>report_IntegerOverflowTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>04-19-2026 03:52</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>04-19-2026 03:56</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>04-20-2026 19:37</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04-20-2026 23:18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04-20-2026 23:24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bank.sol</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>report_Bank.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04-21-2026 02:07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04-21-2026 02:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>22</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bank.sol</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>report_Bank.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:25</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bank.sol</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>report_Bank.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:26</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bank.sol</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>report_Bank.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:28</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>22</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:28</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bank.sol</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>report_Bank.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:31</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>22</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:34</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ReentrancyTest.sol</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>report_ReentrancyTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:42</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>VulnerableTest.sol</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>report_VulnerableTest.sol.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04-21-2026 03:44</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VulnerableTest.sol</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>reentrancy-eth</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>report_VulnerableTest.sol.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>